<commit_message>
Update TruongHuynhAnhTuan AI Log - content updated
</commit_message>
<xml_diff>
--- a/ai_logs/TruongHuynhAnhTuan_ai_log.xlsx
+++ b/ai_logs/TruongHuynhAnhTuan_ai_log.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thanh\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\NHOM_04_LAB211_TicketBooking\ai_logs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDFE56FA-8851-4B7A-BEB8-430C02FFB8E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C1191FE-BC3F-4296-8E53-B336C9BF6F18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -734,9 +734,6 @@
     <t>Test với format ngày khác bị lỗi parse</t>
   </si>
   <si>
-    <t>Thêm try-catch và định dạng chuẩn ISO</t>
-  </si>
-  <si>
     <t>False Execution Claim</t>
   </si>
   <si>
@@ -762,6 +759,9 @@
   </si>
   <si>
     <t>Tự viết logic đồng bộ trong BookingController.</t>
+  </si>
+  <si>
+    <t>Thêm try-catch và định dạng chuẩn ISO.</t>
   </si>
 </sst>
 </file>
@@ -952,20 +952,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1281,7 +1281,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="22" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="20"/>
@@ -1300,7 +1300,7 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -1308,7 +1308,7 @@
         <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -1316,7 +1316,7 @@
         <v>4</v>
       </c>
       <c r="C6" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -1324,7 +1324,7 @@
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -1519,7 +1519,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="22" t="s">
         <v>38</v>
       </c>
       <c r="B1" s="20"/>
@@ -1531,7 +1531,7 @@
       <c r="H1" s="20"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="23" t="s">
         <v>39</v>
       </c>
       <c r="B2" s="20"/>
@@ -2170,7 +2170,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="21" t="s">
         <v>51</v>
       </c>
       <c r="B1" s="20"/>
@@ -2180,7 +2180,7 @@
       <c r="F1" s="20"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="19" t="s">
         <v>52</v>
       </c>
       <c r="B2" s="20"/>
@@ -2256,7 +2256,7 @@
         <v>231</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -2264,19 +2264,19 @@
         <v>21</v>
       </c>
       <c r="B7" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="C7" s="7" t="s">
         <v>233</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="D7" s="7" t="s">
         <v>234</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="E7" s="7" t="s">
         <v>235</v>
       </c>
-      <c r="E7" s="7" t="s">
-        <v>236</v>
-      </c>
       <c r="F7" s="7" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -2507,7 +2507,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="22" t="s">
         <v>78</v>
       </c>
       <c r="B1" s="20"/>
@@ -2515,7 +2515,7 @@
       <c r="D1" s="20"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="24" t="s">
         <v>79</v>
       </c>
       <c r="B2" s="20"/>

</xml_diff>